<commit_message>
Actualiza documentación PLAFT y métricas LexIA
</commit_message>
<xml_diff>
--- a/LexIA_Diario/Comparativo de identificación de normas VF (1).xlsx
+++ b/LexIA_Diario/Comparativo de identificación de normas VF (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://interbankpe-my.sharepoint.com/personal/shernandez2_intercorp_com_pe/Documents/PLAFT/GenIA/Normativo/LexIA_Diario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="330" documentId="11_FF9E2F5B496FDA3AB52BB0B2B6FDBBEC0357B1A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAE6CAA8-09D5-4A19-B12F-52726A29477B}"/>
+  <xr:revisionPtr revIDLastSave="354" documentId="11_FF9E2F5B496FDA3AB52BB0B2B6FDBBEC0357B1A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76C6455B-6FAC-4842-8952-D3366FFEB454}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2479" uniqueCount="968">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2494" uniqueCount="974">
   <si>
     <t>Dia</t>
   </si>
@@ -2900,6 +2900,26 @@
   </si>
   <si>
     <t>Modifican el Reglamento Operativo del Programa Impulso Empresarial MYPE – IMPULSO MYPERU</t>
+  </si>
+  <si>
+    <t>Nº 115-2026-PCM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decreto Supremo que declara el Estado de Emergencia en algunos distritos de las provincias de Huancavelica y Tayacaja del departamento de Huancavelica y de
+las provincias de Chupaca, Concepción y Huancayo del departamento de Junín, por impacto de daños a consecuencia de movimientos sísmicos </t>
+  </si>
+  <si>
+    <t>Nº 116-2026-PCM</t>
+  </si>
+  <si>
+    <t>Decreto Supremo que declara el Estado de Emergencia en varios distritos de algunas provincias de los departamentos de Apurímac, Arequipa, Ayacucho, Cusco,
+Huancavelica, Huánuco, Junín, La Libertad, Loreto, Madre De Dios, Moquegua, Pasco, Puno, San Martín, Tacna y Ucayali, por peligro inminente ante déficit hídrico para el período de lluvias 2026-2027</t>
+  </si>
+  <si>
+    <t>SBS N° 02027-2026</t>
+  </si>
+  <si>
+    <t>Modifican la Resolución SBS N° 04131-2025 y el Reglamento de Notificación vía Casilla Electrónica de la SBS</t>
   </si>
   <si>
     <t>IDENTIFICÓ LA NORMA DE INTERÉS</t>
@@ -13175,6 +13195,66 @@
         <v>941</v>
       </c>
     </row>
+    <row r="464" spans="1:6" ht="57.75">
+      <c r="A464" s="3">
+        <v>46247</v>
+      </c>
+      <c r="B464" t="s">
+        <v>46</v>
+      </c>
+      <c r="C464" t="s">
+        <v>942</v>
+      </c>
+      <c r="D464" t="s">
+        <v>29</v>
+      </c>
+      <c r="E464" t="s">
+        <v>30</v>
+      </c>
+      <c r="F464" s="45" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="465" spans="1:6" ht="87">
+      <c r="A465" s="3">
+        <v>46247</v>
+      </c>
+      <c r="B465" t="s">
+        <v>46</v>
+      </c>
+      <c r="C465" t="s">
+        <v>944</v>
+      </c>
+      <c r="D465" t="s">
+        <v>29</v>
+      </c>
+      <c r="E465" t="s">
+        <v>30</v>
+      </c>
+      <c r="F465" s="45" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="466" spans="1:6">
+      <c r="A466" s="3">
+        <v>46247</v>
+      </c>
+      <c r="B466" t="s">
+        <v>49</v>
+      </c>
+      <c r="C466" t="s">
+        <v>946</v>
+      </c>
+      <c r="D466" t="s">
+        <v>29</v>
+      </c>
+      <c r="E466" t="s">
+        <v>30</v>
+      </c>
+      <c r="F466" s="4" t="s">
+        <v>947</v>
+      </c>
+    </row>
     <row r="1048573" ht="12.75" customHeight="1"/>
     <row r="1048574" ht="12.75" customHeight="1"/>
     <row r="1048575" ht="12.75" customHeight="1"/>
@@ -13199,7 +13279,7 @@
   <sheetData>
     <row r="2" spans="2:8" ht="15" customHeight="1">
       <c r="D2" s="34" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="E2" s="34"/>
     </row>
@@ -13208,10 +13288,10 @@
         <v>21</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
       <c r="E3" s="36" t="s">
         <v>24</v>
@@ -13220,44 +13300,44 @@
         <v>25</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="362.45">
       <c r="B4" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="H4" s="38" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="304.5">
       <c r="B5" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>29</v>
@@ -13269,18 +13349,18 @@
         <v>31</v>
       </c>
       <c r="H5" s="40" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="409.5">
       <c r="B6" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>29</v>
@@ -13292,18 +13372,18 @@
         <v>34</v>
       </c>
       <c r="H6" s="41" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="409.5">
       <c r="B7" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C7" s="16" t="s">
+        <v>961</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>955</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>949</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>29</v>
@@ -13315,15 +13395,15 @@
         <v>37</v>
       </c>
       <c r="H7" s="41" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="409.5">
       <c r="B8" s="12" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="D8" s="42"/>
       <c r="E8" s="12" t="s">
@@ -13339,10 +13419,10 @@
     </row>
     <row r="9" spans="2:8" ht="409.5">
       <c r="B9" s="12" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="D9" s="42"/>
       <c r="E9" s="12" t="s">
@@ -13358,13 +13438,13 @@
     </row>
     <row r="10" spans="2:8" ht="409.5">
       <c r="B10" s="12" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>29</v>
@@ -13379,55 +13459,55 @@
     </row>
     <row r="11" spans="2:8" ht="275.45">
       <c r="B11" s="12" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="H11" s="42"/>
     </row>
     <row r="12" spans="2:8" ht="188.45">
       <c r="B12" s="12" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="40" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="H12" s="42"/>
     </row>
     <row r="13" spans="2:8" ht="409.5">
       <c r="B13" s="12" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>29</v>
@@ -13436,7 +13516,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="H13" s="42"/>
     </row>
@@ -13454,36 +13534,36 @@
   <sheetData>
     <row r="2" spans="2:8" ht="362.45">
       <c r="B2" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="H2" s="38" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="304.5">
       <c r="B3" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>29</v>
@@ -13495,18 +13575,18 @@
         <v>31</v>
       </c>
       <c r="H3" s="40" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="409.5">
       <c r="B4" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>29</v>
@@ -13518,18 +13598,18 @@
         <v>34</v>
       </c>
       <c r="H4" s="41" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="409.5">
       <c r="B5" s="12" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>961</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>955</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>949</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>29</v>
@@ -13541,15 +13621,15 @@
         <v>37</v>
       </c>
       <c r="H5" s="41" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="409.5">
       <c r="B6" s="12" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="D6" s="42"/>
       <c r="E6" s="12" t="s">
@@ -13565,10 +13645,10 @@
     </row>
     <row r="7" spans="2:8" ht="409.5">
       <c r="B7" s="12" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="D7" s="42"/>
       <c r="E7" s="12" t="s">
@@ -13584,13 +13664,13 @@
     </row>
     <row r="8" spans="2:8" ht="409.5">
       <c r="B8" s="12" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>29</v>
@@ -13605,55 +13685,55 @@
     </row>
     <row r="9" spans="2:8" ht="275.45">
       <c r="B9" s="12" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G9" s="40" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="H9" s="42"/>
     </row>
     <row r="10" spans="2:8" ht="188.45">
       <c r="B10" s="12" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="H10" s="42"/>
     </row>
     <row r="11" spans="2:8" ht="409.5">
       <c r="B11" s="12" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>29</v>
@@ -13662,7 +13742,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="H11" s="42"/>
     </row>

</xml_diff>